<commit_message>
feat: add protein length retrieval script and data file
</commit_message>
<xml_diff>
--- a/artifacts/proteins_list.xlsx
+++ b/artifacts/proteins_list.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="48">
   <si>
     <t xml:space="preserve">Protein</t>
   </si>
@@ -34,6 +34,9 @@
     <t xml:space="preserve">Paper 3 (Bioinformatics 2022)</t>
   </si>
   <si>
+    <t xml:space="preserve">Full sequence length</t>
+  </si>
+  <si>
     <t xml:space="preserve">1A7D</t>
   </si>
   <si>
@@ -56,6 +59,9 @@
   </si>
   <si>
     <t xml:space="preserve">1HBE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nan</t>
   </si>
   <si>
     <t xml:space="preserve">1HZ4</t>
@@ -278,7 +284,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:O41"/>
-  <sheetFormatPr defaultColWidth="8.6953125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.70703125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -293,7 +299,9 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1"/>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
@@ -307,18 +315,20 @@
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>118</v>
+      </c>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
@@ -332,18 +342,20 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E3" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>156</v>
+      </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
@@ -357,18 +369,20 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E4" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>144</v>
+      </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
@@ -382,18 +396,20 @@
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E5" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>142</v>
+      </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
@@ -407,18 +423,20 @@
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E6" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>289</v>
+      </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
@@ -432,18 +450,20 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E7" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>13</v>
+      </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
@@ -457,18 +477,20 @@
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E8" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>373</v>
+      </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
@@ -482,18 +504,20 @@
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E9" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>155</v>
+      </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
@@ -507,18 +531,20 @@
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E10" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>122</v>
+      </c>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
@@ -532,18 +558,20 @@
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E11" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>148</v>
+      </c>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
@@ -557,18 +585,20 @@
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E12" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>150</v>
+      </c>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
@@ -582,18 +612,20 @@
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E13" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>245</v>
+      </c>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
@@ -607,18 +639,20 @@
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E14" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>256</v>
+      </c>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
@@ -632,18 +666,20 @@
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E15" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>96</v>
+      </c>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
@@ -657,18 +693,20 @@
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E16" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>345</v>
+      </c>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
@@ -682,18 +720,20 @@
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E17" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>201</v>
+      </c>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
@@ -707,18 +747,20 @@
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E18" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>207</v>
+      </c>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
@@ -732,18 +774,20 @@
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E19" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>585</v>
+      </c>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
@@ -757,18 +801,20 @@
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E20" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>140</v>
+      </c>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
@@ -782,18 +828,20 @@
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E21" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>293</v>
+      </c>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
@@ -807,18 +855,20 @@
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E22" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>6104</v>
+      </c>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
@@ -832,18 +882,20 @@
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E23" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>13</v>
+      </c>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
@@ -857,18 +909,20 @@
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E24" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>329</v>
+      </c>
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
@@ -882,18 +936,20 @@
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E25" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>270</v>
+      </c>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
@@ -907,18 +963,20 @@
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E26" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>7512</v>
+      </c>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
@@ -932,18 +990,20 @@
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E27" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>201</v>
+      </c>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
@@ -957,18 +1017,20 @@
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E28" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>415</v>
+      </c>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
@@ -982,18 +1044,20 @@
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E29" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>1444</v>
+      </c>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
@@ -1007,18 +1071,20 @@
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E30" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>119</v>
+      </c>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
@@ -1032,18 +1098,20 @@
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E31" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>144</v>
+      </c>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
@@ -1057,18 +1125,20 @@
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E32" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>390</v>
+      </c>
       <c r="F32" s="2"/>
       <c r="G32" s="2"/>
       <c r="H32" s="2"/>
@@ -1082,18 +1152,20 @@
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E33" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>204</v>
+      </c>
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
@@ -1107,18 +1179,20 @@
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E34" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>458</v>
+      </c>
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
@@ -1132,18 +1206,20 @@
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E35" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>4136</v>
+      </c>
       <c r="F35" s="2"/>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
@@ -1157,18 +1233,20 @@
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E36" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="E36" s="2" t="n">
+        <v>1850</v>
+      </c>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
@@ -1182,18 +1260,20 @@
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E37" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>349</v>
+      </c>
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
@@ -1207,18 +1287,20 @@
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E38" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>2478</v>
+      </c>
       <c r="F38" s="2"/>
       <c r="G38" s="2"/>
       <c r="H38" s="2"/>
@@ -1232,18 +1314,20 @@
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E39" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>11904</v>
+      </c>
       <c r="F39" s="2"/>
       <c r="G39" s="2"/>
       <c r="H39" s="2"/>
@@ -1257,18 +1341,20 @@
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E40" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="E40" s="2" t="n">
+        <v>1748</v>
+      </c>
       <c r="F40" s="2"/>
       <c r="G40" s="2"/>
       <c r="H40" s="2"/>
@@ -1282,18 +1368,20 @@
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E41" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="E41" s="2" t="n">
+        <v>10847</v>
+      </c>
       <c r="F41" s="2"/>
       <c r="G41" s="2"/>
       <c r="H41" s="2"/>

</xml_diff>

<commit_message>
fix: update proteins length
</commit_message>
<xml_diff>
--- a/artifacts/proteins_list.xlsx
+++ b/artifacts/proteins_list.xlsx
@@ -49,6 +49,9 @@
     <t xml:space="preserve">1BJ7</t>
   </si>
   <si>
+    <t xml:space="preserve">Nan</t>
+  </si>
+  <si>
     <t xml:space="preserve">1BZ4</t>
   </si>
   <si>
@@ -59,9 +62,6 @@
   </si>
   <si>
     <t xml:space="preserve">1HBE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nan</t>
   </si>
   <si>
     <t xml:space="preserve">1HZ4</t>
@@ -253,7 +253,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -264,6 +264,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -284,7 +288,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:O41"/>
-  <sheetFormatPr defaultColWidth="8.70703125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.72265625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -303,8 +307,6 @@
         <v>4</v>
       </c>
       <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -326,12 +328,10 @@
       <c r="D2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" s="0" t="n">
         <v>118</v>
       </c>
       <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
@@ -353,12 +353,10 @@
       <c r="D3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="2" t="n">
-        <v>156</v>
+      <c r="E3" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
@@ -369,7 +367,7 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>6</v>
@@ -380,12 +378,10 @@
       <c r="D4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="0" t="n">
         <v>144</v>
       </c>
       <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
@@ -396,7 +392,7 @@
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>6</v>
@@ -407,12 +403,10 @@
       <c r="D5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="0" t="n">
         <v>142</v>
       </c>
       <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
@@ -423,7 +417,7 @@
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>7</v>
@@ -434,12 +428,10 @@
       <c r="D6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" s="0" t="n">
         <v>289</v>
       </c>
       <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
@@ -450,7 +442,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>7</v>
@@ -461,12 +453,10 @@
       <c r="D7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>13</v>
+      <c r="E7" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
@@ -488,12 +478,10 @@
       <c r="D8" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="0" t="n">
         <v>373</v>
       </c>
       <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
@@ -515,12 +503,10 @@
       <c r="D9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" s="0" t="n">
         <v>155</v>
       </c>
       <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
@@ -542,12 +528,10 @@
       <c r="D10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E10" s="0" t="n">
         <v>122</v>
       </c>
       <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
@@ -569,12 +553,10 @@
       <c r="D11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="E11" s="0" t="n">
         <v>148</v>
       </c>
       <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
@@ -596,12 +578,10 @@
       <c r="D12" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E12" s="2" t="n">
+      <c r="E12" s="0" t="n">
         <v>150</v>
       </c>
       <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
@@ -623,12 +603,10 @@
       <c r="D13" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E13" s="2" t="n">
+      <c r="E13" s="0" t="n">
         <v>245</v>
       </c>
       <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
@@ -650,12 +628,10 @@
       <c r="D14" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E14" s="2" t="n">
+      <c r="E14" s="0" t="n">
         <v>256</v>
       </c>
       <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
@@ -677,12 +653,10 @@
       <c r="D15" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="E15" s="0" t="n">
         <v>96</v>
       </c>
       <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
@@ -704,12 +678,10 @@
       <c r="D16" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E16" s="2" t="n">
+      <c r="E16" s="0" t="n">
         <v>345</v>
       </c>
       <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
@@ -731,12 +703,10 @@
       <c r="D17" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E17" s="2" t="n">
+      <c r="E17" s="0" t="n">
         <v>201</v>
       </c>
       <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
       <c r="K17" s="2"/>
@@ -758,12 +728,10 @@
       <c r="D18" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E18" s="2" t="n">
+      <c r="E18" s="0" t="n">
         <v>207</v>
       </c>
       <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
@@ -785,12 +753,10 @@
       <c r="D19" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E19" s="2" t="n">
+      <c r="E19" s="0" t="n">
         <v>585</v>
       </c>
       <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="2"/>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
@@ -812,12 +778,10 @@
       <c r="D20" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E20" s="2" t="n">
+      <c r="E20" s="0" t="n">
         <v>140</v>
       </c>
       <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-      <c r="H20" s="2"/>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
@@ -839,12 +803,10 @@
       <c r="D21" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E21" s="2" t="n">
+      <c r="E21" s="0" t="n">
         <v>293</v>
       </c>
       <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
-      <c r="H21" s="2"/>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
@@ -866,12 +828,10 @@
       <c r="D22" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E22" s="2" t="n">
-        <v>6104</v>
+      <c r="E22" s="0" t="n">
+        <v>233</v>
       </c>
       <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
-      <c r="H22" s="2"/>
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
@@ -893,12 +853,10 @@
       <c r="D23" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E23" s="2" t="s">
-        <v>13</v>
+      <c r="E23" s="0" t="n">
+        <v>117</v>
       </c>
       <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
@@ -920,12 +878,10 @@
       <c r="D24" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E24" s="2" t="n">
+      <c r="E24" s="0" t="n">
         <v>329</v>
       </c>
       <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-      <c r="H24" s="2"/>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
@@ -947,12 +903,10 @@
       <c r="D25" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E25" s="2" t="n">
+      <c r="E25" s="0" t="n">
         <v>270</v>
       </c>
       <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
@@ -974,12 +928,10 @@
       <c r="D26" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E26" s="2" t="n">
-        <v>7512</v>
+      <c r="E26" s="0" t="n">
+        <v>222</v>
       </c>
       <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="2"/>
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
@@ -1001,12 +953,10 @@
       <c r="D27" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E27" s="2" t="n">
+      <c r="E27" s="0" t="n">
         <v>201</v>
       </c>
       <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
-      <c r="H27" s="2"/>
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
       <c r="K27" s="2"/>
@@ -1028,12 +978,10 @@
       <c r="D28" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E28" s="2" t="n">
+      <c r="E28" s="0" t="n">
         <v>415</v>
       </c>
       <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
-      <c r="H28" s="2"/>
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
@@ -1055,12 +1003,10 @@
       <c r="D29" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E29" s="2" t="n">
-        <v>1444</v>
+      <c r="E29" s="0" t="n">
+        <v>361</v>
       </c>
       <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
       <c r="K29" s="2"/>
@@ -1082,12 +1028,10 @@
       <c r="D30" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E30" s="2" t="n">
+      <c r="E30" s="0" t="n">
         <v>119</v>
       </c>
       <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
-      <c r="H30" s="2"/>
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
       <c r="K30" s="2"/>
@@ -1109,12 +1053,10 @@
       <c r="D31" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E31" s="2" t="n">
+      <c r="E31" s="0" t="n">
         <v>144</v>
       </c>
       <c r="F31" s="2"/>
-      <c r="G31" s="2"/>
-      <c r="H31" s="2"/>
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
       <c r="K31" s="2"/>
@@ -1136,12 +1078,10 @@
       <c r="D32" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E32" s="2" t="n">
-        <v>390</v>
+      <c r="E32" s="0" t="n">
+        <v>102</v>
       </c>
       <c r="F32" s="2"/>
-      <c r="G32" s="2"/>
-      <c r="H32" s="2"/>
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
       <c r="K32" s="2"/>
@@ -1163,12 +1103,10 @@
       <c r="D33" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E33" s="2" t="n">
+      <c r="E33" s="0" t="n">
         <v>204</v>
       </c>
       <c r="F33" s="2"/>
-      <c r="G33" s="2"/>
-      <c r="H33" s="2"/>
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
       <c r="K33" s="2"/>
@@ -1190,12 +1128,10 @@
       <c r="D34" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E34" s="2" t="n">
+      <c r="E34" s="0" t="n">
         <v>458</v>
       </c>
       <c r="F34" s="2"/>
-      <c r="G34" s="2"/>
-      <c r="H34" s="2"/>
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
       <c r="K34" s="2"/>
@@ -1217,12 +1153,10 @@
       <c r="D35" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E35" s="2" t="n">
-        <v>4136</v>
+      <c r="E35" s="0" t="n">
+        <v>1034</v>
       </c>
       <c r="F35" s="2"/>
-      <c r="G35" s="2"/>
-      <c r="H35" s="2"/>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
       <c r="K35" s="2"/>
@@ -1244,12 +1178,10 @@
       <c r="D36" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E36" s="2" t="n">
-        <v>1850</v>
+      <c r="E36" s="0" t="n">
+        <v>439</v>
       </c>
       <c r="F36" s="2"/>
-      <c r="G36" s="2"/>
-      <c r="H36" s="2"/>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
       <c r="K36" s="2"/>
@@ -1271,12 +1203,10 @@
       <c r="D37" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E37" s="2" t="n">
+      <c r="E37" s="0" t="n">
         <v>349</v>
       </c>
       <c r="F37" s="2"/>
-      <c r="G37" s="2"/>
-      <c r="H37" s="2"/>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
       <c r="K37" s="2"/>
@@ -1298,12 +1228,10 @@
       <c r="D38" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E38" s="2" t="n">
-        <v>2478</v>
+      <c r="E38" s="0" t="n">
+        <v>177</v>
       </c>
       <c r="F38" s="2"/>
-      <c r="G38" s="2"/>
-      <c r="H38" s="2"/>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
       <c r="K38" s="2"/>
@@ -1325,12 +1253,10 @@
       <c r="D39" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E39" s="2" t="n">
-        <v>11904</v>
+      <c r="E39" s="0" t="n">
+        <v>291</v>
       </c>
       <c r="F39" s="2"/>
-      <c r="G39" s="2"/>
-      <c r="H39" s="2"/>
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
       <c r="K39" s="2"/>
@@ -1352,12 +1278,10 @@
       <c r="D40" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E40" s="2" t="n">
-        <v>1748</v>
+      <c r="E40" s="0" t="n">
+        <v>327</v>
       </c>
       <c r="F40" s="2"/>
-      <c r="G40" s="2"/>
-      <c r="H40" s="2"/>
       <c r="I40" s="2"/>
       <c r="J40" s="2"/>
       <c r="K40" s="2"/>
@@ -1379,12 +1303,10 @@
       <c r="D41" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E41" s="2" t="n">
-        <v>10847</v>
+      <c r="E41" s="0" t="n">
+        <v>1703</v>
       </c>
       <c r="F41" s="2"/>
-      <c r="G41" s="2"/>
-      <c r="H41" s="2"/>
       <c r="I41" s="2"/>
       <c r="J41" s="2"/>
       <c r="K41" s="2"/>

</xml_diff>